<commit_message>
fix(excel): restore prerequisite order; slug-link all cross-references
Move References into Source & prepare as lesson 0001 (its pre-reorder
position) — the authored order is again a valid topological sort of the
builds_on DAG. Replace all ten stale bare-number prose references with
slug links or 'this lesson' per CONTRACT.md. Drop the soft
sumifs->pivottables edge: its only evidence was a contrast sentence, now
reworded as a neutral forward link. Regenerated pages, index, curriculum
and workbook; CONTRACT.md deviations 2 and 3 marked resolved.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai_training/teach-buying-analyst/excel/artefacts/excel-course-workbook.xlsx
+++ b/ai_training/teach-buying-analyst/excel/artefacts/excel-course-workbook.xlsx
@@ -8,16 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tables" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sort &amp; Filter" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sort &amp; Filter soln" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="Data validation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Data validation soln" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="Text formulas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Text formulas soln" sheetId="8" state="hidden" r:id="rId8"/>
-    <sheet name="Power Query" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Power Query soln" sheetId="10" state="hidden" r:id="rId10"/>
-    <sheet name="References" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="References" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sort &amp; Filter" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sort &amp; Filter soln" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Data validation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Data validation soln" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="Text formulas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Text formulas soln" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet name="Power Query" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Power Query soln" sheetId="11" state="hidden" r:id="rId11"/>
     <sheet name="Logical &amp; IFERROR" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Logical &amp; IFERROR soln" sheetId="13" state="hidden" r:id="rId13"/>
     <sheet name="Aggregation" sheetId="14" state="visible" r:id="rId14"/>
@@ -48,7 +48,7 @@
   <definedNames>
     <definedName name="Rate">'Tables'!$F$1</definedName>
     <definedName name="Revenue">'Named ranges soln'!$B$2:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sort &amp; Filter soln'!$A$1:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sort &amp; Filter soln'!$A$1:$F$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="32">'Print soln'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="32">'Print soln'!$A$1:$F$13</definedName>
   </definedNames>
@@ -719,72 +719,72 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tables</t>
+          <t>References</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lesson 0001 — Tables: the modern foundation</t>
+          <t>Lesson 0001 — Relative &amp; absolute references</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sort &amp; Filter</t>
+          <t>Tables</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lesson 0002 — Sort &amp; Filter: order and isolate</t>
+          <t>Lesson 0002 — Tables: the modern foundation</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Data validation</t>
+          <t>Sort &amp; Filter</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lesson 0003 — Data validation: controlled dropdowns</t>
+          <t>Lesson 0003 — Sort &amp; Filter: order and isolate</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Text formulas</t>
+          <t>Data validation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lesson 0004 — Text formulas: clean &amp; combine</t>
+          <t>Lesson 0004 — Data validation: controlled dropdowns</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Power Query</t>
+          <t>Text formulas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lesson 0005 — Get &amp; Transform (Power Query)</t>
+          <t>Lesson 0005 — Text formulas: clean &amp; combine</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>References</t>
+          <t>Power Query</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lesson 0006 — Relative &amp; absolute references</t>
+          <t>Lesson 0006 — Get &amp; Transform (Power Query)</t>
         </is>
       </c>
     </row>
@@ -962,6 +962,173 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>WEEKLY EXPORT — do not edit above</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Your task</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Category</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cases</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revenue </t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Click a cell in the block, then Data &gt; From Table/Range. In the editor: Remove Top Rows (the title), Use First Row as Headers, Trim the text columns, set Revenue to a number, Remove Blank Rows, then Close &amp; Load. Compare with the 'Power Query soln' tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> stacked chips 12pk 300g</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snacks </t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>120</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3480</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CORN PUFFS 12pk 150g </t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Snacks</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>90</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2232</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> sourdough loaf 800g</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bakery</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2160</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cheddar cheese 500g </t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> DAIRY</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>45</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2205</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> free-range eggs 12pk</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">produce </t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>80</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1952</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F2:J6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1089,167 +1256,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Case cost (GBP)</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Landed cost (AUD)</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Exchange rate (GBP to AUD)</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="n">
-        <v>1.92</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Stacked Chips 12pk 300g</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n">
-        <v>14.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Noodle Snaks 12pk 250g</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Your task</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Rice Crackers 24pk 100g</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>18.75</v>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>In C2 type  =B2*$F$1  then fill down to C11. Change the rate in F1 and watch every row recalculate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Salted Pretzels 16pk 200g</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>9.800000000000001</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Corn Puffs 12pk 150g</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>12.4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Veggie Straws 12pk 120g</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>13.6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Popcorn 10pk 100g</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Cheese Twists 16pk 180g</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>10.9</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Pretzel Bites 20pk 220g</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>15.3</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Tortilla Rounds 12pk 330g</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>16.2</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="E4:H8"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4338,9 +4344,14 @@
           <t>Case cost (GBP)</t>
         </is>
       </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Landed cost (AUD)</t>
+        </is>
+      </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Rate</t>
+          <t>Exchange rate (GBP to AUD)</t>
         </is>
       </c>
       <c r="F1" s="4" t="n">
@@ -4350,21 +4361,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cheddar Cheese 500g</t>
+          <t>Stacked Chips 12pk 300g</t>
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>24.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sourdough Loaf 800g</t>
+          <t>Noodle Snaks 12pk 250g</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>18.75</v>
+        <v>11.2</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
@@ -4375,86 +4386,86 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Free-range Eggs 12pk</t>
+          <t>Rice Crackers 24pk 100g</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>12.2</v>
+        <v>18.75</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Click the data, press Ctrl+T, name it Products on the Table Design tab. Add a Landed cost column:  =[@[Case cost (GBP)]]*Rate  — it fills down by itself.</t>
+          <t>In C2 type  =B2*$F$1  then fill down to C11. Change the rate in F1 and watch every row recalculate.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Salted Butter 250g</t>
+          <t>Salted Pretzels 16pk 200g</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>15.9</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Greek Yoghurt 1kg</t>
+          <t>Corn Puffs 12pk 150g</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>6.4</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Orange Juice 2L</t>
+          <t>Veggie Straws 12pk 120g</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>4.8</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chicken Breast 1kg</t>
+          <t>Popcorn 10pk 100g</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Basmati Rice 5kg</t>
+          <t>Cheese Twists 16pk 180g</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>13.2</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Olive Oil 1L</t>
+          <t>Pretzel Bites 20pk 220g</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>9.75</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dark Chocolate 200g</t>
+          <t>Tortilla Rounds 12pk 330g</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>3.9</v>
+        <v>16.2</v>
       </c>
     </row>
   </sheetData>
@@ -7508,571 +7519,151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Cases</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Revenue (AUD)</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>Your task</t>
-        </is>
+          <t>Case cost (GBP)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="n">
+        <v>1.92</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Acme Foods</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Stacked Chips 12pk 300g</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>120</v>
-      </c>
-      <c r="F2" s="8" t="n">
-        <v>3480</v>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>Press Ctrl+Shift+L to switch on the filter arrows. Open the Revenue (AUD) dropdown and Sort Largest to Smallest, then open the Category dropdown and tick only Snacks. Clear the filter to bring every row back — filtering hides, it never deletes.</t>
-        </is>
+          <t>Cheddar Cheese 500g</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>24.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Acme Foods</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Corn Puffs 12pk 150g</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>90</v>
-      </c>
-      <c r="F3" s="8" t="n">
-        <v>2232</v>
+          <t>Sourdough Loaf 800g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Your task</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Bakery</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>BrightHarvest</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sourdough Loaf 800g</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>60</v>
-      </c>
-      <c r="F4" s="8" t="n">
-        <v>2160</v>
+          <t>Free-range Eggs 12pk</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Click the data, press Ctrl+T, name it Products on the Table Design tab. Add a Landed cost column:  =[@[Case cost (GBP)]]*Rate  — it fills down by itself.</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Coastal Co</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Cheddar Cheese 500g</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>45</v>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>2205</v>
+          <t>Salted Butter 250g</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>15.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Produce</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GreenField</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Free-range Eggs 12pk</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>80</v>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>1952</v>
+          <t>Greek Yoghurt 1kg</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>6.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Acme Foods</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Stacked Chips 12pk 300g</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>140</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>4060</v>
+          <t>Orange Juice 2L</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Harvest Lane</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Rice Crackers 24pk 100g</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>70</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>2625</v>
+          <t>Chicken Breast 1kg</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Bakery</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>BrightHarvest</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Sourdough Loaf 800g</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>75</v>
-      </c>
-      <c r="F9" s="8" t="n">
-        <v>2700</v>
+          <t>Basmati Rice 5kg</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>13.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Coastal Co</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Salted Butter 250g</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>55</v>
-      </c>
-      <c r="F10" s="8" t="n">
-        <v>1749</v>
+          <t>Olive Oil 1L</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>9.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Coastal Co</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Greek Yoghurt 1kg</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>65</v>
-      </c>
-      <c r="F11" s="8" t="n">
-        <v>1248</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Produce</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>GreenField</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Free-range Eggs 12pk</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>95</v>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>2318</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Acme Foods</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Corn Puffs 12pk 150g</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>110</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>2728</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Harvest Lane</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Popcorn 10pk 100g</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>130</v>
-      </c>
-      <c r="F14" s="8" t="n">
-        <v>2210</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Bakery</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>BrightHarvest</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Sourdough Loaf 800g</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>85</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <v>3060</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Coastal Co</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Cheddar Cheese 500g</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>50</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>2450</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Produce</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>GreenField</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Basmati Rice 5kg</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>40</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>1056</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Produce</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>GreenField</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Orange Juice 2L</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>100</v>
-      </c>
-      <c r="F18" s="8" t="n">
-        <v>1920</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Snacks</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Harvest Lane</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Pretzel Bites 20pk 220g</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>60</v>
-      </c>
-      <c r="F19" s="8" t="n">
-        <v>1836</v>
+          <t>Dark Chocolate 200g</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>3.9</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="H2:L6"/>
+    <mergeCell ref="E4:H8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9700,6 +9291,582 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Cases</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Revenue (AUD)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Your task</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Acme Foods</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Stacked Chips 12pk 300g</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>3480</v>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Press Ctrl+Shift+L to switch on the filter arrows. Open the Revenue (AUD) dropdown and Sort Largest to Smallest, then open the Category dropdown and tick only Snacks. Clear the filter to bring every row back — filtering hides, it never deletes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Acme Foods</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Corn Puffs 12pk 150g</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>2232</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bakery</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BrightHarvest</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sourdough Loaf 800g</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Coastal Co</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Cheddar Cheese 500g</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GreenField</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Free-range Eggs 12pk</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>80</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>1952</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Acme Foods</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Stacked Chips 12pk 300g</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>140</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>4060</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Harvest Lane</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rice Crackers 24pk 100g</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>2625</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bakery</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BrightHarvest</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sourdough Loaf 800g</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>75</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Coastal Co</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Salted Butter 250g</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>55</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Coastal Co</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Greek Yoghurt 1kg</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>65</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>1248</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GreenField</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Free-range Eggs 12pk</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>95</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>2318</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Acme Foods</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Corn Puffs 12pk 150g</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>110</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>2728</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Harvest Lane</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Popcorn 10pk 100g</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>130</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bakery</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BrightHarvest</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sourdough Loaf 800g</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>85</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>3060</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Coastal Co</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Cheddar Cheese 500g</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GreenField</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Basmati Rice 5kg</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>40</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GreenField</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Orange Juice 2L</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Harvest Lane</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pretzel Bites 20pk 220g</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>60</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>1836</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="H2:L6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10253,7 +10420,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10464,7 +10631,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10663,7 +10830,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10905,7 +11072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11247,171 +11414,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>WEEKLY EXPORT — do not edit above</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Your task</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Product </t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Category</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Cases</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Revenue </t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Click a cell in the block, then Data &gt; From Table/Range. In the editor: Remove Top Rows (the title), Use First Row as Headers, Trim the text columns, set Revenue to a number, Remove Blank Rows, then Close &amp; Load. Compare with the 'Power Query soln' tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> stacked chips 12pk 300g</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">snacks </t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>120</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>3480</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CORN PUFFS 12pk 150g </t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Snacks</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>90</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2232</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> sourdough loaf 800g</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>bakery</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>60</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2160</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cheddar cheese 500g </t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> DAIRY</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>45</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2205</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> free-range eggs 12pk</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">produce </t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>80</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1952</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="F2:J6"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>